<commit_message>
Stage 8 review fixes: C-023
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/FM20/MV-2026-292/MV-2026-292_AssayWorksheet_092826_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/FM20/MV-2026-292/MV-2026-292_AssayWorksheet_092826_v03.xlsx
@@ -164,7 +164,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Recovery column to be checked on the low-recovery rows before the unbound fraction is quoted</t>
+        <t>Retain recovery with any quoted unbound fraction and check qualifications against the analyte card.</t>
       </text>
     </comment>
   </commentList>
@@ -179,7 +179,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Check the &lt;1 µM result against the QC standard before it goes into the summary</t>
+        <t>Retain the &lt; qualifier when quoting the lower-limit solubility result; final formulation recommendations await the open Caco-2 recovery checks.</t>
       </text>
     </comment>
   </commentList>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MV-2026-292 assay worksheet, interim</t>
+          <t>Merrivoss Bioanalysis Inc, a Tarnovell company | MV-2026-292 assay worksheet, interim</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Compounds tested</t>
+          <t>Study test article count</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -695,34 +695,34 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>FM20-02006</t>
+          <t>Source record</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Caco-2 recovery, low-solubility branch</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Carole Mills</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FM20-02030</t>
+          <t>Caco-2 run records</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Caco-2 recovery, low-solubility branch</t>
+          <t>Recovery checks for the poorly soluble branch</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -735,16 +735,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>FM20-02054</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Carole Mills</t>
-        </is>
-      </c>
+          <t>Accession receipt records</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Confirm matrix-lot mapping</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -780,7 +786,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Human plasma, RED device, 4 h, 37 °C. Rows with low recovery are not used for the unbound fraction until checked.</t>
+          <t>Human plasma, equilibrium dialysis, 4 h, 37 °C. Binding, unbound fraction and recovery are reported together; consult the analyte cards for matrix acceptance qualifications. This table contains the currently recorded subset.</t>
         </is>
       </c>
     </row>

</xml_diff>